<commit_message>
Rediseño login - Mejoras modulo Ble
</commit_message>
<xml_diff>
--- a/quala/CheckListQuala.xlsx
+++ b/quala/CheckListQuala.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karinabanda/Desktop/Proyectos/Reportes/Reportes Diarios/proyecto/quala/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Xaldigital\test\quala\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF80F1A4-3691-5248-B22B-264A22EDD061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A21ADD-B0B2-4148-9156-F4FFC86E8E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -84,9 +84,6 @@
     <t>Free Storage Space Last Hour (GB)</t>
   </si>
   <si>
-    <t>Estado de las alarmas</t>
-  </si>
-  <si>
     <t>Disponibilidad de la página web</t>
   </si>
   <si>
@@ -100,12 +97,15 @@
 * Free Storage Space: Verificación de que el espacio libre en la RDS sea superior a 10 GB.
 Recomendación: No depender únicamente de los comentarios anexados; se sugiere realizar una revisión adicional para mayor precisión.</t>
   </si>
+  <si>
+    <t>Status</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -139,25 +139,32 @@
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="0"/>
       <name val="Aptos Narrow (Cuerpo)"/>
     </font>
     <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,8 +201,14 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="26">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -308,29 +321,6 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -462,75 +452,121 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -751,7 +787,7 @@
   <cols>
     <col min="1" max="1" width="3.6640625" customWidth="1"/>
     <col min="2" max="2" width="39.5" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="8" width="10.5" customWidth="1"/>
     <col min="9" max="10" width="12.33203125" customWidth="1"/>
     <col min="11" max="11" width="11.33203125" customWidth="1"/>
@@ -765,75 +801,75 @@
   <sheetData>
     <row r="1" spans="2:21" ht="15.75" customHeight="1"/>
     <row r="2" spans="2:21" ht="27" customHeight="1">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="35"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="11"/>
     </row>
     <row r="3" spans="2:21" ht="27" customHeight="1">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" s="8"/>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="6" t="s">
         <v>6</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="8"/>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="P3" s="6" t="s">
         <v>9</v>
       </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="8"/>
-      <c r="S3" s="11" t="s">
+      <c r="S3" s="6" t="s">
         <v>10</v>
       </c>
       <c r="T3" s="7"/>
       <c r="U3" s="8"/>
     </row>
     <row r="4" spans="2:21" ht="15.75" customHeight="1">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
@@ -861,8 +897,8 @@
       <c r="M4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
       <c r="P4" s="1" t="s">
         <v>11</v>
       </c>
@@ -999,19 +1035,20 @@
     <row r="14" spans="2:21" ht="15.75" customHeight="1"/>
     <row r="15" spans="2:21" ht="15.75" customHeight="1"/>
     <row r="16" spans="2:21" ht="24.75" customHeight="1">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="8"/>
-      <c r="O16" s="21" t="s">
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="29"/>
+      <c r="L16" s="29"/>
+      <c r="O16" s="14" t="s">
         <v>15</v>
       </c>
       <c r="P16" s="7"/>
@@ -1022,25 +1059,28 @@
       <c r="U16" s="8"/>
     </row>
     <row r="17" spans="2:21" ht="19.5" customHeight="1">
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="7"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="11" t="s">
+      <c r="E17" s="7"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="7"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="11" t="s">
+      <c r="H17" s="7"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="8"/>
-      <c r="O17" s="22"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="8"/>
+      <c r="O17" s="15"/>
       <c r="P17" s="7"/>
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
@@ -1049,35 +1089,36 @@
       <c r="U17" s="8"/>
     </row>
     <row r="18" spans="2:21" ht="15.75" customHeight="1">
-      <c r="B18" s="10"/>
-      <c r="C18" s="1" t="s">
+      <c r="B18" s="17"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O18" s="22"/>
+      <c r="O18" s="15"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
@@ -1086,9 +1127,9 @@
       <c r="U18" s="8"/>
     </row>
     <row r="19" spans="2:21" ht="15.75" customHeight="1">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="25"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1096,7 +1137,8 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
-      <c r="O19" s="22"/>
+      <c r="L19" s="2"/>
+      <c r="O19" s="15"/>
       <c r="P19" s="7"/>
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
@@ -1105,9 +1147,9 @@
       <c r="U19" s="8"/>
     </row>
     <row r="20" spans="2:21" ht="15.75" customHeight="1">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="25"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1115,6 +1157,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
       <c r="O20" s="4"/>
       <c r="P20" s="5"/>
       <c r="Q20" s="5"/>
@@ -1127,157 +1170,144 @@
       <c r="B21" s="3"/>
     </row>
     <row r="23" spans="2:21" ht="22.5" customHeight="1">
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="14"/>
-      <c r="H23" s="15" t="s">
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="20"/>
+      <c r="O23" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="17"/>
+      <c r="P23" s="30"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="30"/>
+      <c r="S23" s="30"/>
+      <c r="T23" s="30"/>
+      <c r="U23" s="31"/>
     </row>
     <row r="24" spans="2:21" ht="15.75" customHeight="1">
-      <c r="B24" s="22"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="20"/>
-    </row>
-    <row r="25" spans="2:21" ht="15.75" customHeight="1"/>
-    <row r="27" spans="2:21" ht="24.75" customHeight="1">
-      <c r="O27" s="21" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="42"/>
+      <c r="O24" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="7"/>
-      <c r="S27" s="7"/>
-      <c r="T27" s="7"/>
-      <c r="U27" s="8"/>
+      <c r="P24" s="32"/>
+      <c r="Q24" s="32"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="32"/>
+      <c r="T24" s="32"/>
+      <c r="U24" s="33"/>
+    </row>
+    <row r="25" spans="2:21" ht="15.75" customHeight="1">
+      <c r="O25" s="34"/>
+      <c r="P25" s="35"/>
+      <c r="Q25" s="35"/>
+      <c r="R25" s="35"/>
+      <c r="S25" s="35"/>
+      <c r="T25" s="35"/>
+      <c r="U25" s="36"/>
+    </row>
+    <row r="26" spans="2:21" ht="15" customHeight="1">
+      <c r="O26" s="34"/>
+      <c r="P26" s="35"/>
+      <c r="Q26" s="35"/>
+      <c r="R26" s="35"/>
+      <c r="S26" s="35"/>
+      <c r="T26" s="35"/>
+      <c r="U26" s="36"/>
+    </row>
+    <row r="27" spans="2:21" ht="14.5" customHeight="1">
+      <c r="O27" s="34"/>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="35"/>
+      <c r="R27" s="35"/>
+      <c r="S27" s="35"/>
+      <c r="T27" s="35"/>
+      <c r="U27" s="36"/>
     </row>
     <row r="28" spans="2:21" ht="15.75" customHeight="1">
-      <c r="O28" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="26"/>
-      <c r="S28" s="26"/>
-      <c r="T28" s="26"/>
-      <c r="U28" s="27"/>
+      <c r="O28" s="34"/>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="35"/>
+      <c r="R28" s="35"/>
+      <c r="S28" s="35"/>
+      <c r="T28" s="35"/>
+      <c r="U28" s="36"/>
     </row>
     <row r="29" spans="2:21" ht="15.75" customHeight="1">
-      <c r="O29" s="28"/>
-      <c r="P29" s="29"/>
-      <c r="Q29" s="29"/>
-      <c r="R29" s="29"/>
-      <c r="S29" s="29"/>
-      <c r="T29" s="29"/>
-      <c r="U29" s="30"/>
+      <c r="O29" s="34"/>
+      <c r="P29" s="35"/>
+      <c r="Q29" s="35"/>
+      <c r="R29" s="35"/>
+      <c r="S29" s="35"/>
+      <c r="T29" s="35"/>
+      <c r="U29" s="36"/>
     </row>
     <row r="30" spans="2:21" ht="15.75" customHeight="1">
-      <c r="O30" s="28"/>
-      <c r="P30" s="29"/>
-      <c r="Q30" s="29"/>
-      <c r="R30" s="29"/>
-      <c r="S30" s="29"/>
-      <c r="T30" s="29"/>
-      <c r="U30" s="30"/>
+      <c r="O30" s="34"/>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="35"/>
+      <c r="R30" s="35"/>
+      <c r="S30" s="35"/>
+      <c r="T30" s="35"/>
+      <c r="U30" s="36"/>
     </row>
     <row r="31" spans="2:21" ht="15.75" customHeight="1">
-      <c r="O31" s="28"/>
-      <c r="P31" s="29"/>
-      <c r="Q31" s="29"/>
-      <c r="R31" s="29"/>
-      <c r="S31" s="29"/>
-      <c r="T31" s="29"/>
-      <c r="U31" s="30"/>
+      <c r="O31" s="34"/>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="35"/>
+      <c r="R31" s="35"/>
+      <c r="S31" s="35"/>
+      <c r="T31" s="35"/>
+      <c r="U31" s="36"/>
     </row>
     <row r="32" spans="2:21" ht="15.75" customHeight="1">
-      <c r="O32" s="28"/>
-      <c r="P32" s="29"/>
-      <c r="Q32" s="29"/>
-      <c r="R32" s="29"/>
-      <c r="S32" s="29"/>
-      <c r="T32" s="29"/>
-      <c r="U32" s="30"/>
+      <c r="O32" s="34"/>
+      <c r="P32" s="35"/>
+      <c r="Q32" s="35"/>
+      <c r="R32" s="35"/>
+      <c r="S32" s="35"/>
+      <c r="T32" s="35"/>
+      <c r="U32" s="36"/>
     </row>
     <row r="33" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O33" s="28"/>
-      <c r="P33" s="29"/>
-      <c r="Q33" s="29"/>
-      <c r="R33" s="29"/>
-      <c r="S33" s="29"/>
-      <c r="T33" s="29"/>
-      <c r="U33" s="30"/>
+      <c r="O33" s="34"/>
+      <c r="P33" s="35"/>
+      <c r="Q33" s="35"/>
+      <c r="R33" s="35"/>
+      <c r="S33" s="35"/>
+      <c r="T33" s="35"/>
+      <c r="U33" s="36"/>
     </row>
     <row r="34" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O34" s="28"/>
-      <c r="P34" s="29"/>
-      <c r="Q34" s="29"/>
-      <c r="R34" s="29"/>
-      <c r="S34" s="29"/>
-      <c r="T34" s="29"/>
-      <c r="U34" s="30"/>
+      <c r="O34" s="34"/>
+      <c r="P34" s="35"/>
+      <c r="Q34" s="35"/>
+      <c r="R34" s="35"/>
+      <c r="S34" s="35"/>
+      <c r="T34" s="35"/>
+      <c r="U34" s="36"/>
     </row>
     <row r="35" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O35" s="28"/>
-      <c r="P35" s="29"/>
-      <c r="Q35" s="29"/>
-      <c r="R35" s="29"/>
-      <c r="S35" s="29"/>
-      <c r="T35" s="29"/>
-      <c r="U35" s="30"/>
-    </row>
-    <row r="36" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O36" s="28"/>
-      <c r="P36" s="29"/>
-      <c r="Q36" s="29"/>
-      <c r="R36" s="29"/>
-      <c r="S36" s="29"/>
-      <c r="T36" s="29"/>
-      <c r="U36" s="30"/>
-    </row>
-    <row r="37" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O37" s="28"/>
-      <c r="P37" s="29"/>
-      <c r="Q37" s="29"/>
-      <c r="R37" s="29"/>
-      <c r="S37" s="29"/>
-      <c r="T37" s="29"/>
-      <c r="U37" s="30"/>
-    </row>
-    <row r="38" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O38" s="28"/>
-      <c r="P38" s="29"/>
-      <c r="Q38" s="29"/>
-      <c r="R38" s="29"/>
-      <c r="S38" s="29"/>
-      <c r="T38" s="29"/>
-      <c r="U38" s="30"/>
-    </row>
-    <row r="39" spans="15:21" ht="15.75" customHeight="1">
-      <c r="O39" s="31"/>
-      <c r="P39" s="32"/>
-      <c r="Q39" s="32"/>
-      <c r="R39" s="32"/>
-      <c r="S39" s="32"/>
-      <c r="T39" s="32"/>
-      <c r="U39" s="33"/>
-    </row>
+      <c r="O35" s="37"/>
+      <c r="P35" s="38"/>
+      <c r="Q35" s="38"/>
+      <c r="R35" s="38"/>
+      <c r="S35" s="38"/>
+      <c r="T35" s="38"/>
+      <c r="U35" s="39"/>
+    </row>
+    <row r="36" spans="15:21" ht="15.75" customHeight="1"/>
+    <row r="37" spans="15:21" ht="15.75" customHeight="1"/>
+    <row r="38" spans="15:21" ht="15.75" customHeight="1"/>
+    <row r="39" spans="15:21" ht="15.75" customHeight="1"/>
     <row r="40" spans="15:21" ht="15.75" customHeight="1"/>
     <row r="41" spans="15:21" ht="15.75" customHeight="1"/>
     <row r="42" spans="15:21" ht="15.75" customHeight="1"/>
@@ -2244,7 +2274,21 @@
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="25">
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="O23:U23"/>
+    <mergeCell ref="O24:U35"/>
+    <mergeCell ref="O16:U16"/>
+    <mergeCell ref="O17:U17"/>
+    <mergeCell ref="O18:U18"/>
+    <mergeCell ref="O19:U19"/>
     <mergeCell ref="P3:R3"/>
     <mergeCell ref="S3:U3"/>
     <mergeCell ref="B2:U2"/>
@@ -2256,21 +2300,6 @@
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="O3:O4"/>
-    <mergeCell ref="O16:U16"/>
-    <mergeCell ref="O17:U17"/>
-    <mergeCell ref="O18:U18"/>
-    <mergeCell ref="O19:U19"/>
-    <mergeCell ref="O28:U39"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="H23:M23"/>
-    <mergeCell ref="H24:M24"/>
-    <mergeCell ref="O27:U27"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B16:K16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="I17:K17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>